<commit_message>
Teplica A: KEF Q350 pairs + active sub on Volta LIVE 4.400
- Variant A reworked (folder renamed to A-kef-volta-sub): CM82 out A
  feeds Volta LIVE 4.400 (ch1/ch2: KEF Q350 pairs at 4 ohm, ch3:
  Radiotehnika Alfa 1.04 MKII active sub via high-level input, ch4
  spare); street + restroom on CA1202 100 V; CRC-V per zone (hall on
  CM82 out A, street on CA1202 "A+B", restroom on CA1202 "B").
- Facts from the CA/CM quick start guides: per-channel RJ45 pinout,
  common front master on CA, CM82 priority inputs A/E, rack brackets
  included (rack-kit lines dropped from estimates).
- Estimate rebuilt: A ~468k, B ~192k, C ~372k (+140k optional sub).
- New A schematic, BOM; comparison, variant C checks, summary updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpptGYyvFpUmP2Tbj75fbk
</commit_message>
<xml_diff>
--- a/sound/smeta-teplica.xlsx
+++ b/sound/smeta-teplica.xlsx
@@ -500,11 +500,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Вариант A — Lab.gruppen, винтаж + сабвуфер</t>
+          <t>Вариант A — KEF Q350 + активный сабвуфер (Volta + CA1202)</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <f>'Вариант A'!G23</f>
+        <f>'Вариант A'!G20</f>
         <v/>
       </c>
       <c r="C5" s="3" t="n"/>
@@ -530,11 +530,11 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>'Вариант C'!G19</f>
+        <f>'Вариант C'!G18</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>'Вариант C'!G26</f>
+        <f>'Вариант C'!G24</f>
         <v/>
       </c>
       <c r="D7" s="3">
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Вариант A — Lab.gruppen, винтаж + сабвуфер</t>
+          <t>Вариант A — KEF Q350 + активный сабвуфер (Volta + CA1202)</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA1202 — зал, две пары (4/8 Ом)</t>
+          <t>Volta LIVE 4.400 — зал: 2 пары KEF + сабвуфер</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>50000</v>
+        <v>25984</v>
       </c>
       <c r="G6" s="6">
         <f>E6*F6</f>
@@ -688,7 +688,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>45–60 тыс.; для NS-10M — CA602 ≈ 40–50 тыс.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA2401 — сабвуфер (8 Ом)</t>
+          <t>Lab.gruppen CA1202 — улица + туалет (100 В)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>43–60 тыс.</t>
+          <t>45–60 тыс.; крепёж в комплекте</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA2402 — улица + туалет (100 В)</t>
+          <t>Lab.gruppen CRC-VEU — регулятор зоны</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>60000</v>
+        <v>6500</v>
       </c>
       <c r="G8" s="6">
         <f>E8*F8</f>
@@ -758,7 +758,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>51–69 тыс.; можно CA1202 (−10 тыс.)</t>
+          <t>Pult.ru 6 510</t>
         </is>
       </c>
     </row>
@@ -773,19 +773,19 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Комплект монтажа двух ½ 19" в 1U</t>
+          <t>Рамка на 3 поста + подрозетники</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="G9" s="6">
         <f>E9*F9</f>
@@ -793,7 +793,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>оценка, уточнить артикул</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -803,24 +803,24 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Оборудование</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CRC-VEU — регулятор зоны</t>
+          <t>KEF Q350 — полочная акустика, пара</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>пара</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>6500</v>
+        <v>39000</v>
       </c>
       <c r="G10" s="6">
         <f>E10*F10</f>
@@ -828,7 +828,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru 6 510</t>
+          <t>цена заказчика</t>
         </is>
       </c>
     </row>
@@ -838,24 +838,24 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Оборудование</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Рамка на 3 поста + подрозетники</t>
+          <t>Radiotehnika Alfa 1.04 MKII — активный сабвуфер 10″</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>1500</v>
+        <v>49990</v>
       </c>
       <c r="G11" s="6">
         <f>E11*F11</f>
@@ -863,7 +863,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>Audiomania</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Винтажные hi-fi колонки зала (б/у)</t>
+          <t>CVGaudio OSR608TBL — улица, 100 В / 30 Вт, IP65</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -887,10 +887,10 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>17500</v>
+        <v>9622</v>
       </c>
       <c r="G12" s="6">
         <f>E12*F12</f>
@@ -898,7 +898,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>бюджет 15–20 тыс. за шт.</t>
+          <t>цена из сметы В.О.</t>
         </is>
       </c>
     </row>
@@ -913,19 +913,19 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Резерв на ревизию б/у колонок (подвесы, твитеры)</t>
+          <t>CVGaudio NF4TBL — туалет, 100 В / 8 Вт</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>10000</v>
+        <v>5933</v>
       </c>
       <c r="G13" s="6">
         <f>E13*F13</f>
@@ -933,7 +933,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>цена из сметы В.О.</t>
         </is>
       </c>
     </row>
@@ -943,12 +943,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Оборудование</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Сабвуфер Tannoy VSX 10BP</t>
+          <t>Музыкальный плеер / стример с линейным выходом</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -960,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>80000</v>
+        <v>15000</v>
       </c>
       <c r="G14" s="6">
         <f>E14*F14</f>
@@ -968,7 +968,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>оценка по цене в США (~$800); бюджетный 10" 8 Ом — от ~40 тыс.</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -978,24 +978,24 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Монтаж</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>CVGaudio OSR608TBL — улица, 100 В / 30 Вт, IP65</t>
+          <t>Шкаф 19″ 9U + блок розеток + полка + перфопанель</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>9622</v>
+        <v>20000</v>
       </c>
       <c r="G15" s="6">
         <f>E15*F15</f>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -1013,24 +1013,24 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Монтаж</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>CVGaudio NF4TBL — туалет, 100 В / 8 Вт</t>
+          <t>Кабель: 2×2,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>5933</v>
+        <v>25000</v>
       </c>
       <c r="G16" s="6">
         <f>E16*F16</f>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>оценка, по длине трасс</t>
         </is>
       </c>
     </row>
@@ -1048,24 +1048,24 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Оборудование</t>
+          <t>Монтаж</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Музыкальный плеер / стример с линейным выходом</t>
+          <t>Кронштейны для KEF, тросики, расходные материалы</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="G17" s="6">
         <f>E17*F17</f>
@@ -1083,24 +1083,24 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Монтаж</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Шкаф 19" 9U + блок розеток + полка + перфопанель</t>
+          <t>Монтаж кабеля, колонок, шкафа; ПНР</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>20000</v>
+        <v>90000</v>
       </c>
       <c r="G18" s="6">
         <f>E18*F18</f>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>оценка по смете В.О. (45 тыс. за простую систему)</t>
         </is>
       </c>
     </row>
@@ -1118,24 +1118,24 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Монтаж</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Кабель: 2×2,5 (зал, саб), 2×1,5 (100 В, улица), Cat5e ×3</t>
+          <t>Транспортные расходы</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>25000</v>
+        <v>5000</v>
       </c>
       <c r="G19" s="6">
         <f>E19*F19</f>
@@ -1143,131 +1143,26 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>оценка, по длине трасс</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Монтаж</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Расходные материалы, кронштейны для колонок, тросики</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>12000</v>
-      </c>
-      <c r="G20" s="6">
-        <f>E20*F20</f>
-        <v/>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Монтаж кабеля, колонок, шкафа; ПНР</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>90000</v>
-      </c>
-      <c r="G21" s="6">
-        <f>E21*F21</f>
-        <v/>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>оценка по смете В.О. (45 тыс. за простую систему)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Транспортные расходы</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G22" s="6">
-        <f>E22*F22</f>
-        <v/>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="8">
-        <f>SUM(G5:G22)</f>
-        <v/>
-      </c>
-      <c r="H23" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="8">
+        <f>SUM(G5:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1797,7 +1692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1982,7 +1877,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Комплект монтажа двух ½ 19" в 1U</t>
+          <t>Lab.gruppen CRC-VEU — регулятор зоны</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1991,10 +1886,10 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>5000</v>
+        <v>6500</v>
       </c>
       <c r="G8" s="6">
         <f>E8*F8</f>
@@ -2002,7 +1897,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>Pult.ru 6 510</t>
         </is>
       </c>
     </row>
@@ -2017,19 +1912,19 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CRC-VEU — регулятор зоны</t>
+          <t>Рамка на 3 поста + подрозетники</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>6500</v>
+        <v>1500</v>
       </c>
       <c r="G9" s="6">
         <f>E9*F9</f>
@@ -2037,7 +1932,7 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru 6 510</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -2047,24 +1942,24 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Оборудование</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Рамка на 3 поста + подрозетники</t>
+          <t>CVGaudio OSR608TBL — зал 4 шт (30 Вт) + улица 2 шт (20 Вт)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>1500</v>
+        <v>9622</v>
       </c>
       <c r="G10" s="6">
         <f>E10*F10</f>
@@ -2072,7 +1967,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>цена из сметы В.О.</t>
         </is>
       </c>
     </row>
@@ -2087,7 +1982,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>CVGaudio OSR608TBL — зал 4 шт (30 Вт) + улица 2 шт (20 Вт)</t>
+          <t>CVGaudio NF4TBL — туалет, 100 В / 8 Вт</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -2096,10 +1991,10 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>9622</v>
+        <v>5933</v>
       </c>
       <c r="G11" s="6">
         <f>E11*F11</f>
@@ -2117,12 +2012,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Оборудование</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>CVGaudio NF4TBL — туалет, 100 В / 8 Вт</t>
+          <t>Музыкальный плеер / стример с линейным выходом</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -2131,10 +2026,10 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>5933</v>
+        <v>15000</v>
       </c>
       <c r="G12" s="6">
         <f>E12*F12</f>
@@ -2142,7 +2037,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -2152,17 +2047,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Оборудование</t>
+          <t>Монтаж</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Музыкальный плеер / стример с линейным выходом</t>
+          <t>Шкаф 19" 6U + блок розеток + полка</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
@@ -2192,7 +2087,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Шкаф 19" 6U + блок розеток + полка</t>
+          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2204,7 +2099,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="G14" s="6">
         <f>E14*F14</f>
@@ -2212,7 +2107,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>оценка, трасса под саб — сразу</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2122,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
+          <t>Расходные материалы</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -2239,7 +2134,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>18000</v>
+        <v>8000</v>
       </c>
       <c r="G15" s="6">
         <f>E15*F15</f>
@@ -2247,7 +2142,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>оценка, трасса под саб — сразу</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -2257,24 +2152,24 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Монтаж</t>
+          <t>Работы</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Расходные материалы</t>
+          <t>Монтаж кабеля, колонок, шкафа; ПНР</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>8000</v>
+        <v>75000</v>
       </c>
       <c r="G16" s="6">
         <f>E16*F16</f>
@@ -2297,7 +2192,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Монтаж кабеля, колонок, шкафа; ПНР</t>
+          <t>Транспортные расходы</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -2309,7 +2204,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>75000</v>
+        <v>5000</v>
       </c>
       <c r="G17" s="6">
         <f>E17*F17</f>
@@ -2322,61 +2217,40 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Транспортные расходы</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G18" s="6">
-        <f>E18*F18</f>
-        <v/>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="8">
+        <f>SUM(G5:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
       <c r="B19" s="5" t="n"/>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>ИТОГО</t>
-        </is>
-      </c>
+      <c r="C19" s="5" t="n"/>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="6" t="n"/>
-      <c r="G19" s="8">
-        <f>SUM(G5:G18)</f>
-        <v/>
-      </c>
+      <c r="G19" s="6" t="n"/>
       <c r="H19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
       <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Опция: сабвуфер</t>
+        </is>
+      </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="6" t="n"/>
@@ -2384,22 +2258,43 @@
       <c r="H20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="A21" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Опция: сабвуфер</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="5" t="n"/>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Lab.gruppen CA2401 — сабвуфер (8 Ом)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G21" s="6">
+        <f>E21*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>43–60 тыс.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
@@ -2408,7 +2303,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA2401 — сабвуфер (8 Ом)</t>
+          <t>Сабвуфер Tannoy VSX 10BP</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2420,7 +2315,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>50000</v>
+        <v>80000</v>
       </c>
       <c r="G22" s="6">
         <f>E22*F22</f>
@@ -2428,13 +2323,13 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>43–60 тыс.</t>
+          <t>оценка; бюджетный 10" 8 Ом — от ~40 тыс.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
@@ -2443,19 +2338,19 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Сабвуфер Tannoy VSX 10BP</t>
+          <t>Монтаж и настройка сабвуфера</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>80000</v>
+        <v>10000</v>
       </c>
       <c r="G23" s="6">
         <f>E23*F23</f>
@@ -2463,96 +2358,26 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>оценка; бюджетный 10" 8 Ом — от ~40 тыс.</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Опция: сабвуфер</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Комплект монтажа ½ 19" (второй)</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G24" s="6">
-        <f>E24*F24</f>
-        <v/>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Опция: сабвуфер</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Монтаж и настройка сабвуфера</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G25" s="6">
-        <f>E25*F25</f>
-        <v/>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>ИТОГО опция</t>
         </is>
       </c>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="8">
-        <f>SUM(G22:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="8">
+        <f>SUM(G21:G23)</f>
+        <v/>
+      </c>
+      <c r="H24" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Teplica estimates: equipment only, Pult.ru prices; A uses CA602
- Drop labor and transport from all estimates.
- Prices taken from Pult.ru product cards where available (CM82,
  CA602/CA1202/CA2401, CRC-VEU, Volta LIVE 4.400, CVGaudio items,
  Tannoy VSX10 BP, WiiM Pro, 9U cabinet); remaining items marked as
  estimates. Totals: A ~375k, B ~137k, C ~302k (+121k optional sub).
- Variant A: street + restroom on CA602 (street taps 20 W, 40 W of
  60 W); README, BOM and schematic updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpptGYyvFpUmP2Tbj75fbk
</commit_message>
<xml_diff>
--- a/sound/smeta-teplica.xlsx
+++ b/sound/smeta-teplica.xlsx
@@ -500,11 +500,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Вариант A — KEF Q350 + активный сабвуфер (Volta + CA1202)</t>
+          <t>Вариант A — KEF Q350 + активный сабвуфер (Volta + CA602)</t>
         </is>
       </c>
       <c r="B5" s="3">
-        <f>'Вариант A'!G20</f>
+        <f>'Вариант A'!G19</f>
         <v/>
       </c>
       <c r="C5" s="3" t="n"/>
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>'Вариант B'!G17</f>
+        <f>'Вариант B'!G15</f>
         <v/>
       </c>
       <c r="C6" s="3" t="n"/>
@@ -530,11 +530,11 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>'Вариант C'!G18</f>
+        <f>'Вариант C'!G17</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>'Вариант C'!G24</f>
+        <f>'Вариант C'!G22</f>
         <v/>
       </c>
       <c r="D7" s="3">
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Вариант A — KEF Q350 + активный сабвуфер (Volta + CA1202)</t>
+          <t>Вариант A — KEF Q350 + активный сабвуфер (Volta + CA602)</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>45000</v>
+        <v>45071</v>
       </c>
       <c r="G5" s="6">
         <f>E5*F5</f>
@@ -653,7 +653,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru / VISmedia ≈ 45 тыс.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>25984</v>
+        <v>31626</v>
       </c>
       <c r="G6" s="6">
         <f>E6*F6</f>
@@ -688,7 +688,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
+          <t>Pult.ru, в наличии (встречалась и 25 984)</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA1202 — улица + туалет (100 В)</t>
+          <t>Lab.gruppen CA602 — улица + туалет (2 × 60 Вт, 100 В)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -715,7 +715,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>50000</v>
+        <v>35330</v>
       </c>
       <c r="G7" s="6">
         <f>E7*F7</f>
@@ -723,7 +723,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>45–60 тыс.; крепёж в комплекте</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
         <v>3</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>6500</v>
+        <v>6510</v>
       </c>
       <c r="G8" s="6">
         <f>E8*F8</f>
@@ -758,7 +758,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru 6 510</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>цена заказчика</t>
+          <t>цена заказчика (Pult.ru: 45 500)</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Audiomania</t>
+          <t>Audiomania (на Pult.ru нет)</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>CVGaudio OSR608TBL — улица, 100 В / 30 Вт, IP65</t>
+          <t>CVGaudio OSR608TBL — улица, 100 В / 20 Вт, IP65</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -890,7 +890,7 @@
         <v>2</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>9622</v>
+        <v>9417</v>
       </c>
       <c r="G12" s="6">
         <f>E12*F12</f>
@@ -898,7 +898,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>5933</v>
+        <v>6150</v>
       </c>
       <c r="G13" s="6">
         <f>E13*F13</f>
@@ -933,7 +933,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Музыкальный плеер / стример с линейным выходом</t>
+          <t>Сетевой плеер WiiM Pro</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -960,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>15000</v>
+        <v>22999</v>
       </c>
       <c r="G14" s="6">
         <f>E14*F14</f>
@@ -968,7 +968,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -983,19 +983,19 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Шкаф 19″ 9U + блок розеток + полка + перфопанель</t>
+          <t>Шкаф настенный 19″ 9U (Wize Pro W9U45R)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>20000</v>
+        <v>17535</v>
       </c>
       <c r="G15" s="6">
         <f>E15*F15</f>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Кабель: 2×2,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
+          <t>Блок розеток 19″ с выключателем + полка 1U</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1030,7 +1030,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>25000</v>
+        <v>5000</v>
       </c>
       <c r="G16" s="6">
         <f>E16*F16</f>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>оценка, по длине трасс</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Кронштейны для KEF, тросики, расходные материалы</t>
+          <t>Кабель: 2×2,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>12000</v>
+        <v>25000</v>
       </c>
       <c r="G17" s="6">
         <f>E17*F17</f>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>оценка, по длине трасс</t>
         </is>
       </c>
     </row>
@@ -1083,24 +1083,24 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Монтаж</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Монтаж кабеля, колонок, шкафа; ПНР</t>
+          <t>Кронштейны для KEF, тросики, расходные материалы</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>90000</v>
+        <v>12000</v>
       </c>
       <c r="G18" s="6">
         <f>E18*F18</f>
@@ -1108,61 +1108,26 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>оценка по смете В.О. (45 тыс. за простую систему)</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Транспортные расходы</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G19" s="6">
-        <f>E19*F19</f>
-        <v/>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="8">
-        <f>SUM(G5:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="8">
+        <f>SUM(G5:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1175,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1255,7 +1220,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>CVGaudio REBOX-T18 — 180 Вт / 100 В, MP3/FM/BT</t>
+          <t>CVGaudio REBOX-T18 V.2 — 180 Вт / 100 В, MP3/FM/BT</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1267,7 +1232,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>35226</v>
+        <v>35269</v>
       </c>
       <c r="G5" s="6">
         <f>E5*F5</f>
@@ -1275,7 +1240,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1275,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>cvg.ru</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1310,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>cvg.ru; можно VA-160, если 60 Вт подтвердится</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1337,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>2500</v>
+        <v>2393</v>
       </c>
       <c r="G8" s="6">
         <f>E8*F8</f>
@@ -1380,7 +1345,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1407,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>9622</v>
+        <v>9417</v>
       </c>
       <c r="G10" s="6">
         <f>E10*F10</f>
@@ -1450,7 +1415,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1442,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>5933</v>
+        <v>6150</v>
       </c>
       <c r="G11" s="6">
         <f>E11*F11</f>
@@ -1485,7 +1450,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1595,91 +1560,21 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Монтаж кабеля, колонок, регуляторов; ПНР</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G15" s="6">
-        <f>E15*F15</f>
-        <v/>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>оценка по смете В.О.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Транспортные расходы</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>3300</v>
-      </c>
-      <c r="G16" s="6">
-        <f>E16*F16</f>
-        <v/>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>как в смете В.О.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="8">
-        <f>SUM(G5:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="8">
+        <f>SUM(G5:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1692,7 +1587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1784,7 +1679,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>45000</v>
+        <v>45071</v>
       </c>
       <c r="G5" s="6">
         <f>E5*F5</f>
@@ -1792,7 +1687,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru / VISmedia ≈ 45 тыс.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1714,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>50000</v>
+        <v>50100</v>
       </c>
       <c r="G6" s="6">
         <f>E6*F6</f>
@@ -1827,7 +1722,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>43–60 тыс.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1749,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>50000</v>
+        <v>44996</v>
       </c>
       <c r="G7" s="6">
         <f>E7*F7</f>
@@ -1862,7 +1757,7 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>45–60 тыс.</t>
+          <t>Pult.ru (встречалась 42 502)</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1784,7 @@
         <v>3</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>6500</v>
+        <v>6510</v>
       </c>
       <c r="G8" s="6">
         <f>E8*F8</f>
@@ -1897,7 +1792,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru 6 510</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1854,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>9622</v>
+        <v>9417</v>
       </c>
       <c r="G10" s="6">
         <f>E10*F10</f>
@@ -1967,7 +1862,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1889,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>5933</v>
+        <v>6150</v>
       </c>
       <c r="G11" s="6">
         <f>E11*F11</f>
@@ -2002,7 +1897,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>цена из сметы В.О.</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -2017,7 +1912,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Музыкальный плеер / стример с линейным выходом</t>
+          <t>Сетевой плеер WiiM Pro</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -2029,7 +1924,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>15000</v>
+        <v>22999</v>
       </c>
       <c r="G12" s="6">
         <f>E12*F12</f>
@@ -2037,7 +1932,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -2052,19 +1947,19 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Шкаф 19" 6U + блок розеток + полка</t>
+          <t>Шкаф настенный 19″ 9U (Wize Pro W9U45R)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>15000</v>
+        <v>17535</v>
       </c>
       <c r="G13" s="6">
         <f>E13*F13</f>
@@ -2072,7 +1967,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>Pult.ru</t>
         </is>
       </c>
     </row>
@@ -2087,7 +1982,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
+          <t>Блок розеток 19″ с выключателем + полка 1U</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2099,7 +1994,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>18000</v>
+        <v>5000</v>
       </c>
       <c r="G14" s="6">
         <f>E14*F14</f>
@@ -2107,7 +2002,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>оценка, трасса под саб — сразу</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2017,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Расходные материалы</t>
+          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -2134,7 +2029,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>8000</v>
+        <v>18000</v>
       </c>
       <c r="G15" s="6">
         <f>E15*F15</f>
@@ -2142,7 +2037,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>оценка, трасса под саб — сразу</t>
         </is>
       </c>
     </row>
@@ -2152,24 +2047,24 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Работы</t>
+          <t>Монтаж</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Монтаж кабеля, колонок, шкафа; ПНР</t>
+          <t>Расходные материалы</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>75000</v>
+        <v>8000</v>
       </c>
       <c r="G16" s="6">
         <f>E16*F16</f>
@@ -2182,61 +2077,40 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Работы</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Транспортные расходы</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G17" s="6">
-        <f>E17*F17</f>
-        <v/>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="8">
+        <f>SUM(G5:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
       <c r="B18" s="5" t="n"/>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>ИТОГО</t>
-        </is>
-      </c>
+      <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="6" t="n"/>
-      <c r="G18" s="8">
-        <f>SUM(G5:G17)</f>
-        <v/>
-      </c>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
       <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Опция: сабвуфер</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="6" t="n"/>
@@ -2244,22 +2118,43 @@
       <c r="H19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="A20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Опция: сабвуфер</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="5" t="n"/>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Lab.gruppen CA2401 — сабвуфер (8 Ом)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>50100</v>
+      </c>
+      <c r="G20" s="6">
+        <f>E20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -2268,7 +2163,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA2401 — сабвуфер (8 Ом)</t>
+          <t>Сабвуфер Tannoy VSX10 BP</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -2280,7 +2175,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>50000</v>
+        <v>71340</v>
       </c>
       <c r="G21" s="6">
         <f>E21*F21</f>
@@ -2288,96 +2183,26 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>43–60 тыс.</t>
+          <t>Pult.ru (чёрный; белый бывает со скидкой ~58 690)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Опция: сабвуфер</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Сабвуфер Tannoy VSX 10BP</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>80000</v>
-      </c>
-      <c r="G22" s="6">
-        <f>E22*F22</f>
-        <v/>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>оценка; бюджетный 10" 8 Ом — от ~40 тыс.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Опция: сабвуфер</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Монтаж и настройка сабвуфера</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G23" s="6">
-        <f>E23*F23</f>
-        <v/>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>ИТОГО опция</t>
         </is>
       </c>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="8">
-        <f>SUM(G21:G23)</f>
-        <v/>
-      </c>
-      <c r="H24" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="8">
+        <f>SUM(G20:G21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Teplica: variant A2 (KEF Q150), subwoofer optional in A and A2
- A2 = A with KEF Q150 (29 000 per pair, Audiomania promo): README,
  BOM, schematic.
- Subwoofer moved to an option in A and A2 (Volta ch3 and cable laid
  anyway): A 264 046 (+sub 314 036), A2 244 046 (+sub 294 036).
- PDF rebuilt (13 pages): four variants, sub options, Q150 added to
  the size comparison; overview, estimate mirror and summary updated.
  The Google Sheet itself was not changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpptGYyvFpUmP2Tbj75fbk
</commit_message>
<xml_diff>
--- a/sound/smeta-teplica.xlsx
+++ b/sound/smeta-teplica.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Вариант A: KEF Q350 + активный сабвуфер (Volta LIVE 4.400 + CA602)</t>
+          <t>Вариант A: KEF Q350 на Volta LIVE 4.400 + CA602, сабвуфер опционально</t>
         </is>
       </c>
       <c r="B3" s="3" t="n"/>
@@ -568,7 +568,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Volta LIVE 4.400, зал: 2 пары KEF + сабвуфер</t>
+          <t>Volta LIVE 4.400, зал: 2 пары KEF (кан. 3 — под сабвуфер)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
+          <t>CVGaudio OSR608TBL, улица, 100 В / 20 Вт, IP65</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -816,7 +816,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>49990</v>
+        <v>9417</v>
       </c>
       <c r="G12">
         <f>E12*F12</f>
@@ -824,14 +824,10 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Audiomania</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>на Pult.ru нет</t>
-        </is>
-      </c>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -844,7 +840,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CVGaudio OSR608TBL, улица, 100 В / 20 Вт, IP65</t>
+          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -853,10 +849,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>9417</v>
+        <v>6150</v>
       </c>
       <c r="G13">
         <f>E13*F13</f>
@@ -864,10 +860,14 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>CVG</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>есть в наличии</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -875,12 +875,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Шкаф</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -889,10 +889,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>6150</v>
+        <v>17869</v>
       </c>
       <c r="G14">
         <f>E14*F14</f>
@@ -900,14 +900,10 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>есть в наличии</t>
-        </is>
-      </c>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -915,12 +911,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Шкаф</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
+          <t>Блок розеток 19″ 1U с выключателем</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -932,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>17869</v>
+        <v>1755</v>
       </c>
       <c r="G15">
         <f>E15*F15</f>
@@ -940,10 +936,14 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Gembird MAX19-EH8</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -956,7 +956,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Блок розеток 19″ 1U с выключателем</t>
+          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -968,7 +968,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1755</v>
+        <v>2278</v>
       </c>
       <c r="G16">
         <f>E16*F16</f>
@@ -976,12 +976,12 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>ВсеИнструменты</t>
+          <t>Ozon</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Gembird MAX19-EH8</t>
+          <t>под iPad</t>
         </is>
       </c>
     </row>
@@ -991,37 +991,33 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Коммутация</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+          <t>Кабель: 2×1,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2278</v>
+        <v>20000</v>
       </c>
       <c r="G17">
         <f>E17*F17</f>
         <v/>
       </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>Ozon</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>под iPad</t>
+          <t>примерно, нужен расчёт длины трасс</t>
         </is>
       </c>
     </row>
@@ -1031,12 +1027,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Коммутация</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Кабель: 2×1,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
+          <t>Кронштейны для KEF, расходные материалы</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1048,275 +1044,204 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>20000</v>
+        <v>12000</v>
       </c>
       <c r="G18">
         <f>E18*F18</f>
         <v/>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>примерно, нужен расчёт длины трасс</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Шкаф и материалы</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Кронштейны для KEF, расходные материалы</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" t="n">
-        <v>12000</v>
-      </c>
-      <c r="G19">
-        <f>E19*F19</f>
-        <v/>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="G20" s="4">
-        <f>SUM(G5:G19)</f>
-        <v/>
-      </c>
+      <c r="G19" s="4">
+        <f>SUM(G5:G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Вариант A: опция «сабвуфер»</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Вариант B: CVGaudio 100 В, самый простой (один M-123Tm)</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Опция</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>49990</v>
+      </c>
+      <c r="G23">
+        <f>E23*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Audiomania</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>к каналу 3 Volta, розетка 230 В</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G24" s="4">
+        <f>SUM(G23:G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Вариант A2: то же с KEF Q150, сабвуфер опционально</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Раздел</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Цена, ₽</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>Сумма, ₽</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Где купить</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>CVGaudio M-123Tm, микшер-усилитель 120 Вт / 100 В, MP3/FM/BT</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" t="n">
-        <v>43206</v>
-      </c>
-      <c r="G24">
-        <f>E24*F24</f>
-        <v/>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>все три зоны</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>CVGaudio VA-1100, регулятор «Зал» (100 Вт)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" t="n">
-        <v>4246</v>
-      </c>
-      <c r="G25">
-        <f>E25*F25</f>
-        <v/>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>3</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>CVGaudio VA-1100, регулятор «Улица» (100 Вт)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" t="n">
-        <v>4246</v>
-      </c>
-      <c r="G26">
-        <f>E26*F26</f>
-        <v/>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>4</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>CVGaudio VA-110, регулятор «Туалет» (10 Вт)</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" t="n">
-        <v>2393</v>
-      </c>
-      <c r="G27">
-        <f>E27*F27</f>
-        <v/>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1325,34 +1250,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Рамка / подрозетники под регуляторы</t>
+          <t>Lab.gruppen CM82, микшер 8×2</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>1500</v>
+        <v>45071</v>
       </c>
       <c r="G28">
         <f>E28*F28</f>
         <v/>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1361,7 +1286,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>iPad</t>
+          <t>Volta LIVE 4.400, зал: 2 пары KEF (кан. 3 — под сабвуфер)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1373,26 +1298,26 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>25000</v>
+        <v>31626</v>
       </c>
       <c r="G29">
         <f>E29*F29</f>
         <v/>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Авито</t>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>диапазон 17–25 тыс.</t>
+          <t>в наличии; встречалась цена 25 984</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1401,43 +1326,47 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Кабель/адаптер iPad → RCA</t>
+          <t>Lab.gruppen CA602, улица + туалет (2 × 60 Вт, 100 В)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>2000</v>
+        <v>35330</v>
       </c>
       <c r="G30">
         <f>E30*F30</f>
         <v/>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>оценка; или встроенный плеер</t>
+          <t>есть в наличии</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+          <t>Lab.gruppen CRC-VEU, регулятор зоны</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1446,10 +1375,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>2278</v>
+        <v>6510</v>
       </c>
       <c r="G31">
         <f>E31*F31</f>
@@ -1457,63 +1386,63 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>Pult.ru</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>под iPad</t>
+          <t>зал, улица, туалет</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Шкаф</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
+          <t>Рамка на 3 поста + подрозетники</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>17869</v>
+        <v>1500</v>
       </c>
       <c r="G32">
         <f>E32*F32</f>
         <v/>
       </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>оценка</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CVGaudio OSR608TBL, зал 4 шт + улица 1 шт, 100 В</t>
+          <t>iPad</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1522,25 +1451,29 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>9417</v>
+        <v>25000</v>
       </c>
       <c r="G33">
         <f>E33*F33</f>
         <v/>
       </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Авито</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>диапазон 17–25 тыс.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1549,19 +1482,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+          <t>KEF Q150, полочная акустика (пара)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>пара</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
-        <v>6150</v>
+        <v>29000</v>
       </c>
       <c r="G34">
         <f>E34*F34</f>
@@ -1569,356 +1502,360 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>CVG</t>
+          <t>Audiomania</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>есть в наличии</t>
+          <t>акция на Аудиомании (было 52 000)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Кабель 2×1,5 (100 В), уличный кабель</t>
+          <t>CVGaudio OSR608TBL, улица, 100 В / 20 Вт, IP65</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>20000</v>
+        <v>9417</v>
       </c>
       <c r="G35">
         <f>E35*F35</f>
         <v/>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>примерно, нужен расчёт длины трасс</t>
-        </is>
-      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Расходные материалы (крепёж, коробки IP65)</t>
+          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>7000</v>
+        <v>6150</v>
       </c>
       <c r="G36">
         <f>E36*F36</f>
         <v/>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>CVG</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>есть в наличии</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="G37" s="4">
-        <f>SUM(G24:G36)</f>
-        <v/>
+      <c r="A37" t="n">
+        <v>10</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Шкаф</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>17869</v>
+      </c>
+      <c r="G37">
+        <f>E37*F37</f>
+        <v/>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>11</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Блок розеток 19″ 1U с выключателем</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1755</v>
+      </c>
+      <c r="G38">
+        <f>E38*F38</f>
+        <v/>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Gembird MAX19-EH8</t>
+        </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Вариант C: Lab.gruppen 100 В (CA2401 + CA602), сабвуфер опционально</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
+      <c r="A39" t="n">
+        <v>12</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G39">
+        <f>E39*F39</f>
+        <v/>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>под iPad</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Наименование</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>Цена, ₽</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>Сумма, ₽</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>Где купить</t>
-        </is>
-      </c>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>Примечание</t>
+      <c r="A40" t="n">
+        <v>13</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Коммутация</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Кабель: 2×1,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G40">
+        <f>E40*F40</f>
+        <v/>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>примерно, нужен расчёт длины трасс</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Lab.gruppen CM82, микшер 8×2</t>
+          <t>Кронштейны для KEF, расходные материалы</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E41" t="n">
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>45071</v>
+        <v>12000</v>
       </c>
       <c r="G41">
         <f>E41*F41</f>
         <v/>
       </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="n">
-        <v>2</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Lab.gruppen CA2401, зал (100 В)</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" t="n">
-        <v>50100</v>
-      </c>
-      <c r="G42">
-        <f>E42*F42</f>
-        <v/>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>3</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Lab.gruppen CA602, улица + туалет (100 В)</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" t="n">
-        <v>44996</v>
-      </c>
-      <c r="G43">
-        <f>E43*F43</f>
-        <v/>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>есть в наличии</t>
-        </is>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G42" s="4">
+        <f>SUM(G28:G41)</f>
+        <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
-        <v>4</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Lab.gruppen CRC-VEU, регулятор зоны</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>3</v>
-      </c>
-      <c r="F44" t="n">
-        <v>6510</v>
-      </c>
-      <c r="G44">
-        <f>E44*F44</f>
-        <v/>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>зал, улица, туалет</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Вариант A2: опция «сабвуфер»</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
+      <c r="I44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" t="n">
-        <v>5</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Рамка на 3 поста + подрозетники</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G45">
-        <f>E45*F45</f>
-        <v/>
-      </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>оценка</t>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Опция</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>iPad</t>
+          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1930,183 +1867,108 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>25000</v>
+        <v>49990</v>
       </c>
       <c r="G46">
         <f>E46*F46</f>
         <v/>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Авито</t>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>Audiomania</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>диапазон 17–25 тыс.</t>
+          <t>к каналу 3 Volta, розетка 230 В</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
-        <v>7</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Акустика</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>CVGaudio OSR608TBL, зал 4 шт (30 Вт) + улица 1 шт (20 Вт)</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>5</v>
-      </c>
-      <c r="F47" t="n">
-        <v>9417</v>
-      </c>
-      <c r="G47">
-        <f>E47*F47</f>
-        <v/>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>8</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Акустика</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" t="n">
-        <v>6150</v>
-      </c>
-      <c r="G48">
-        <f>E48*F48</f>
-        <v/>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>есть в наличии</t>
-        </is>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G47" s="4">
+        <f>SUM(G46:G46)</f>
+        <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
-        <v>9</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Шкаф</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" t="n">
-        <v>17869</v>
-      </c>
-      <c r="G49">
-        <f>E49*F49</f>
-        <v/>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Вариант B: CVGaudio 100 В, самый простой (один M-123Tm)</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n"/>
+      <c r="C49" s="3" t="n"/>
+      <c r="D49" s="3" t="n"/>
+      <c r="E49" s="3" t="n"/>
+      <c r="F49" s="3" t="n"/>
+      <c r="G49" s="3" t="n"/>
+      <c r="H49" s="3" t="n"/>
+      <c r="I49" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" t="n">
-        <v>10</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Шкаф и материалы</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Блок розеток 19″ 1U с выключателем MDX PDU-8E-10A-Sw</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" t="n">
-        <v>2080</v>
-      </c>
-      <c r="G50">
-        <f>E50*F50</f>
-        <v/>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+          <t>CVGaudio M-123Tm, микшер-усилитель 120 Вт / 100 В, MP3/FM/BT</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2118,7 +1980,7 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>2278</v>
+        <v>43206</v>
       </c>
       <c r="G51">
         <f>E51*F51</f>
@@ -2126,172 +1988,247 @@
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>под iPad</t>
+          <t>все три зоны</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
+          <t>CVGaudio VA-1100, регулятор «Зал» (100 Вт)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E52" t="n">
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>20000</v>
+        <v>4246</v>
       </c>
       <c r="G52">
         <f>E52*F52</f>
         <v/>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>примерно, нужен расчёт длины трасс</t>
-        </is>
-      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Расходные материалы</t>
+          <t>CVGaudio VA-1100, регулятор «Улица» (100 Вт)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E53" t="n">
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>8000</v>
+        <v>4246</v>
       </c>
       <c r="G53">
         <f>E53*F53</f>
         <v/>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>4</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CVGaudio VA-110, регулятор «Туалет» (10 Вт)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>2393</v>
+      </c>
+      <c r="G54">
+        <f>E54*F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>5</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Рамка / подрозетники под регуляторы</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G55">
+        <f>E55*F55</f>
+        <v/>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
         <is>
           <t>оценка</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="G54" s="4">
-        <f>SUM(G41:G53)</f>
-        <v/>
-      </c>
-    </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Вариант C: опция «сабвуфер»</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="n"/>
-      <c r="C56" s="3" t="n"/>
-      <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="n"/>
-      <c r="F56" s="3" t="n"/>
-      <c r="G56" s="3" t="n"/>
-      <c r="H56" s="3" t="n"/>
-      <c r="I56" s="3" t="n"/>
+      <c r="A56" t="n">
+        <v>6</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>iPad</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G56">
+        <f>E56*F56</f>
+        <v/>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Авито</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>диапазон 17–25 тыс.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>Наименование</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>Цена, ₽</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>Сумма, ₽</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>Где купить</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>Примечание</t>
+      <c r="A57" t="n">
+        <v>7</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Кабель/адаптер iPad → RCA</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G57">
+        <f>E57*F57</f>
+        <v/>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>оценка; или встроенный плеер</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Опция</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Усилитель мощности Behringer KM750</t>
+          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2303,7 +2240,7 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>21475</v>
+        <v>2278</v>
       </c>
       <c r="G58">
         <f>E58*F58</f>
@@ -2311,27 +2248,27 @@
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
+          <t>Ozon</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>канал под сабвуфер</t>
+          <t>под iPad</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Опция</t>
+          <t>Шкаф</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
+          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2343,7 +2280,7 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>49990</v>
+        <v>17869</v>
       </c>
       <c r="G59">
         <f>E59*F59</f>
@@ -2351,19 +2288,873 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>10</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CVGaudio OSR608TBL, зал 4 шт + улица 1 шт, 100 В</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>5</v>
+      </c>
+      <c r="F60" t="n">
+        <v>9417</v>
+      </c>
+      <c r="G60">
+        <f>E60*F60</f>
+        <v/>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>11</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>6150</v>
+      </c>
+      <c r="G61">
+        <f>E61*F61</f>
+        <v/>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>CVG</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>есть в наличии</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>12</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Кабель 2×1,5 (100 В), уличный кабель</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G62">
+        <f>E62*F62</f>
+        <v/>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>примерно, нужен расчёт длины трасс</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>13</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Расходные материалы (крепёж, коробки IP65)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G63">
+        <f>E63*F63</f>
+        <v/>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G64" s="4">
+        <f>SUM(G51:G63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Вариант C: Lab.gruppen 100 В (CA2401 + CA602), сабвуфер опционально</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="n"/>
+      <c r="H66" s="3" t="n"/>
+      <c r="I66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>1</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Lab.gruppen CM82, микшер 8×2</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>45071</v>
+      </c>
+      <c r="G68">
+        <f>E68*F68</f>
+        <v/>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Lab.gruppen CA2401, зал (100 В)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>50100</v>
+      </c>
+      <c r="G69">
+        <f>E69*F69</f>
+        <v/>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>3</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Lab.gruppen CA602, улица + туалет (100 В)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>44996</v>
+      </c>
+      <c r="G70">
+        <f>E70*F70</f>
+        <v/>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>есть в наличии</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>4</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Lab.gruppen CRC-VEU, регулятор зоны</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>3</v>
+      </c>
+      <c r="F71" t="n">
+        <v>6510</v>
+      </c>
+      <c r="G71">
+        <f>E71*F71</f>
+        <v/>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>зал, улица, туалет</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>5</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Рамка на 3 поста + подрозетники</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G72">
+        <f>E72*F72</f>
+        <v/>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>оценка</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>6</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>iPad</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G73">
+        <f>E73*F73</f>
+        <v/>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Авито</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>диапазон 17–25 тыс.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>7</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CVGaudio OSR608TBL, зал 4 шт (30 Вт) + улица 1 шт (20 Вт)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>5</v>
+      </c>
+      <c r="F74" t="n">
+        <v>9417</v>
+      </c>
+      <c r="G74">
+        <f>E74*F74</f>
+        <v/>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>8</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>6150</v>
+      </c>
+      <c r="G75">
+        <f>E75*F75</f>
+        <v/>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>CVG</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>есть в наличии</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>9</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Шкаф</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="n">
+        <v>17869</v>
+      </c>
+      <c r="G76">
+        <f>E76*F76</f>
+        <v/>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>10</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Блок розеток 19″ 1U с выключателем MDX PDU-8E-10A-Sw</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="n">
+        <v>2080</v>
+      </c>
+      <c r="G77">
+        <f>E77*F77</f>
+        <v/>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>11</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G78">
+        <f>E78*F78</f>
+        <v/>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>под iPad</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>12</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G79">
+        <f>E79*F79</f>
+        <v/>
+      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>примерно, нужен расчёт длины трасс</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>13</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Расходные материалы</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G80">
+        <f>E80*F80</f>
+        <v/>
+      </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>оценка</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G81" s="4">
+        <f>SUM(G68:G80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Вариант C: опция «сабвуфер»</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="n"/>
+      <c r="C83" s="3" t="n"/>
+      <c r="D83" s="3" t="n"/>
+      <c r="E83" s="3" t="n"/>
+      <c r="F83" s="3" t="n"/>
+      <c r="G83" s="3" t="n"/>
+      <c r="H83" s="3" t="n"/>
+      <c r="I83" s="3" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>1</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Опция</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Усилитель мощности Behringer KM750</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="n">
+        <v>21475</v>
+      </c>
+      <c r="G85">
+        <f>E85*F85</f>
+        <v/>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>канал под сабвуфер</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>2</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Опция</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" t="n">
+        <v>49990</v>
+      </c>
+      <c r="G86">
+        <f>E86*F86</f>
+        <v/>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
           <t>Audiomania</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="C60" s="4" t="inlineStr">
+      <c r="I86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="G60" s="4">
-        <f>SUM(G58:G59)</f>
+      <c r="G87" s="4">
+        <f>SUM(G85:G86)</f>
         <v/>
       </c>
     </row>
@@ -2379,26 +3170,37 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Teplica estimates: add DKC cable channel, end caps and flat corner to all variants (not in PDF)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpptGYyvFpUmP2Tbj75fbk
</commit_message>
<xml_diff>
--- a/sound/smeta-teplica.xlsx
+++ b/sound/smeta-teplica.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1054,310 +1054,310 @@
       <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="C19" s="4" t="inlineStr">
+      <c r="A19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Кабель-канал DKC TA-GN 100×60 (01786), 2 м, под iPad и регуляторы, с перегородкой</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1150</v>
+      </c>
+      <c r="G19">
+        <f>E19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>перегородку и силовой выключатель уточнить, цена по выдаче поиска</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Заглушки DKC LAN 100×60 (00874), 2 шт</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>191</v>
+      </c>
+      <c r="G20">
+        <f>E20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Угол плоский DKC NPAN 100×60 (01745), поворот канала от шкафа к iPad</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>250</v>
+      </c>
+      <c r="G21">
+        <f>E21*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>цена ориентировочно, уточнить</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="G19" s="4">
-        <f>SUM(G5:G18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="G22" s="4">
+        <f>SUM(G5:G21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Вариант A: опция «сабвуфер»</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Раздел</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Цена, ₽</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>Сумма, ₽</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Где купить</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Опция</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" t="n">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
         <v>49990</v>
       </c>
-      <c r="G23">
-        <f>E23*F23</f>
-        <v/>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="G26">
+        <f>E26*F26</f>
+        <v/>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>Audiomania</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>к каналу 3 Volta, розетка 230 В</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="C24" s="4" t="inlineStr">
+    <row r="27">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="G24" s="4">
-        <f>SUM(G23:G23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="G27" s="4">
+        <f>SUM(G26:G26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Вариант A2: то же с KEF Q150, сабвуфер опционально</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Раздел</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>Цена, ₽</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>Сумма, ₽</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>Где купить</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>Примечание</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Lab.gruppen CM82, микшер 8×2</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" t="n">
-        <v>45071</v>
-      </c>
-      <c r="G28">
-        <f>E28*F28</f>
-        <v/>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Volta LIVE 4.400, зал: 2 пары KEF (кан. 3 — под сабвуфер)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" t="n">
-        <v>31626</v>
-      </c>
-      <c r="G29">
-        <f>E29*F29</f>
-        <v/>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>в наличии; встречалась цена 25 984</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>3</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Lab.gruppen CA602, улица + туалет (2 × 60 Вт, 100 В)</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="n">
-        <v>35330</v>
-      </c>
-      <c r="G30">
-        <f>E30*F30</f>
-        <v/>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>есть в наличии</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Lab.gruppen CRC-VEU, регулятор зоны</t>
+          <t>Lab.gruppen CM82, микшер 8×2</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1375,10 +1375,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>6510</v>
+        <v>45071</v>
       </c>
       <c r="G31">
         <f>E31*F31</f>
@@ -1389,15 +1389,11 @@
           <t>Pult.ru</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>зал, улица, туалет</t>
-        </is>
-      </c>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1406,34 +1402,38 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Рамка на 3 поста + подрозетники</t>
+          <t>Volta LIVE 4.400, зал: 2 пары KEF (кан. 3 — под сабвуфер)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>1500</v>
+        <v>31626</v>
       </c>
       <c r="G32">
         <f>E32*F32</f>
         <v/>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>в наличии; встречалась цена 25 984</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>iPad</t>
+          <t>Lab.gruppen CA602, улица + туалет (2 × 60 Вт, 100 В)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1451,50 +1451,50 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>25000</v>
+        <v>35330</v>
       </c>
       <c r="G33">
         <f>E33*F33</f>
         <v/>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Авито</t>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>диапазон 17–25 тыс.</t>
+          <t>есть в наличии</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KEF Q150, полочная акустика (пара)</t>
+          <t>Lab.gruppen CRC-VEU, регулятор зоны</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>пара</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>29000</v>
+        <v>6510</v>
       </c>
       <c r="G34">
         <f>E34*F34</f>
@@ -1502,63 +1502,63 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Audiomania</t>
+          <t>Pult.ru</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>акция на Аудиомании (было 52 000)</t>
+          <t>зал, улица, туалет</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CVGaudio OSR608TBL, улица, 100 В / 20 Вт, IP65</t>
+          <t>Рамка на 3 поста + подрозетники</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>9417</v>
+        <v>1500</v>
       </c>
       <c r="G35">
         <f>E35*F35</f>
         <v/>
       </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>оценка</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+          <t>iPad</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1567,50 +1567,50 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>6150</v>
+        <v>25000</v>
       </c>
       <c r="G36">
         <f>E36*F36</f>
         <v/>
       </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>CVG</t>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Авито</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>есть в наличии</t>
+          <t>диапазон 17–25 тыс.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Шкаф</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
+          <t>KEF Q150, полочная акустика (пара)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>пара</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>17869</v>
+        <v>29000</v>
       </c>
       <c r="G37">
         <f>E37*F37</f>
@@ -1618,23 +1618,27 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr"/>
+          <t>Audiomania</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>акция на Аудиомании (было 52 000)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Блок розеток 19″ 1U с выключателем</t>
+          <t>CVGaudio OSR608TBL, улица, 100 В / 20 Вт, IP65</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1646,7 +1650,7 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>1755</v>
+        <v>9417</v>
       </c>
       <c r="G38">
         <f>E38*F38</f>
@@ -1654,27 +1658,23 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>ВсеИнструменты</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Gembird MAX19-EH8</t>
-        </is>
-      </c>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Акустика</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1683,10 +1683,10 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>2278</v>
+        <v>6150</v>
       </c>
       <c r="G39">
         <f>E39*F39</f>
@@ -1694,54 +1694,54 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Ozon</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>под iPad</t>
+          <t>есть в наличии</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Коммутация</t>
+          <t>Шкаф</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Кабель: 2×1,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
+          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E40" t="n">
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>20000</v>
+        <v>17869</v>
       </c>
       <c r="G40">
         <f>E40*F40</f>
         <v/>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>примерно, нужен расчёт длины трасс</t>
-        </is>
-      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1750,124 +1750,207 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Кронштейны для KEF, расходные материалы</t>
+          <t>Блок розеток 19″ 1U с выключателем</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E41" t="n">
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>12000</v>
+        <v>1755</v>
       </c>
       <c r="G41">
         <f>E41*F41</f>
         <v/>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Gembird MAX19-EH8</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="G42" s="4">
-        <f>SUM(G28:G41)</f>
-        <v/>
+      <c r="A42" t="n">
+        <v>12</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G42">
+        <f>E42*F42</f>
+        <v/>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>под iPad</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>13</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Коммутация</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Кабель: 2×1,5 (пары), 2×1,5 (саб, 100 В), уличный, Cat5e ×3</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G43">
+        <f>E43*F43</f>
+        <v/>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>примерно, нужен расчёт длины трасс</t>
+        </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Вариант A2: опция «сабвуфер»</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="n"/>
-      <c r="C44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n"/>
-      <c r="I44" s="3" t="n"/>
+      <c r="A44" t="n">
+        <v>14</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Кронштейны для KEF, расходные материалы</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G44">
+        <f>E44*F44</f>
+        <v/>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Наименование</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Цена, ₽</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>Сумма, ₽</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>Где купить</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Примечание</t>
+      <c r="A45" t="n">
+        <v>15</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Кабель-канал DKC TA-GN 100×60 (01786), 2 м, под iPad и регуляторы, с перегородкой</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1150</v>
+      </c>
+      <c r="G45">
+        <f>E45*F45</f>
+        <v/>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>перегородку и силовой выключатель уточнить, цена по выдаче поиска</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Опция</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
+          <t>Заглушки DKC LAN 100×60 (00874), 2 шт</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E46" t="n">
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>49990</v>
+        <v>191</v>
       </c>
       <c r="G46">
         <f>E46*F46</f>
@@ -1875,140 +1958,136 @@
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>Audiomania</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>к каналу 3 Volta, розетка 230 В</t>
-        </is>
-      </c>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="C47" s="4" t="inlineStr">
+      <c r="A47" t="n">
+        <v>17</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Угол плоский DKC NPAN 100×60 (01745), поворот канала от шкафа к iPad</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>250</v>
+      </c>
+      <c r="G47">
+        <f>E47*F47</f>
+        <v/>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>цена ориентировочно, уточнить</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="G47" s="4">
-        <f>SUM(G46:G46)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Вариант B: CVGaudio 100 В, самый простой (один M-123Tm)</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="n"/>
-      <c r="C49" s="3" t="n"/>
-      <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
-      <c r="F49" s="3" t="n"/>
-      <c r="G49" s="3" t="n"/>
-      <c r="H49" s="3" t="n"/>
-      <c r="I49" s="3" t="n"/>
+      <c r="G48" s="4">
+        <f>SUM(G31:G47)</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Вариант A2: опция «сабвуфер»</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n"/>
+      <c r="C50" s="3" t="n"/>
+      <c r="D50" s="3" t="n"/>
+      <c r="E50" s="3" t="n"/>
+      <c r="F50" s="3" t="n"/>
+      <c r="G50" s="3" t="n"/>
+      <c r="H50" s="3" t="n"/>
+      <c r="I50" s="3" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Раздел</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>Цена, ₽</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>Сумма, ₽</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>Где купить</t>
         </is>
       </c>
-      <c r="I50" s="4" t="inlineStr">
+      <c r="I51" s="4" t="inlineStr">
         <is>
           <t>Примечание</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>CVGaudio M-123Tm, микшер-усилитель 120 Вт / 100 В, MP3/FM/BT</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" t="n">
-        <v>43206</v>
-      </c>
-      <c r="G51">
-        <f>E51*F51</f>
-        <v/>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>все три зоны</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Опция</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CVGaudio VA-1100, регулятор «Зал» (100 Вт)</t>
+          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2020,7 +2099,7 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>4246</v>
+        <v>49990</v>
       </c>
       <c r="G52">
         <f>E52*F52</f>
@@ -2028,162 +2107,91 @@
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
+          <t>Audiomania</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>к каналу 3 Volta, розетка 230 В</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" t="n">
-        <v>3</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>CVGaudio VA-1100, регулятор «Улица» (100 Вт)</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E53" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" t="n">
-        <v>4246</v>
-      </c>
-      <c r="G53">
-        <f>E53*F53</f>
-        <v/>
-      </c>
-      <c r="H53" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>4</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>CVGaudio VA-110, регулятор «Туалет» (10 Вт)</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" t="n">
-        <v>2393</v>
-      </c>
-      <c r="G54">
-        <f>E54*F54</f>
-        <v/>
-      </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr"/>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G53" s="4">
+        <f>SUM(G52:G52)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" t="n">
-        <v>5</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Рамка / подрозетники под регуляторы</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G55">
-        <f>E55*F55</f>
-        <v/>
-      </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>оценка</t>
-        </is>
-      </c>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Вариант B: CVGaudio 100 В, самый простой (один M-123Tm)</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n"/>
+      <c r="C55" s="3" t="n"/>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="3" t="n"/>
+      <c r="F55" s="3" t="n"/>
+      <c r="G55" s="3" t="n"/>
+      <c r="H55" s="3" t="n"/>
+      <c r="I55" s="3" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" t="n">
-        <v>6</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>iPad</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E56" t="n">
-        <v>1</v>
-      </c>
-      <c r="F56" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G56">
-        <f>E56*F56</f>
-        <v/>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Авито</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>диапазон 17–25 тыс.</t>
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -2192,43 +2200,47 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Кабель/адаптер iPad → RCA</t>
+          <t>CVGaudio M-123Tm, микшер-усилитель 120 Вт / 100 В, MP3/FM/BT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E57" t="n">
         <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>2000</v>
+        <v>43206</v>
       </c>
       <c r="G57">
         <f>E57*F57</f>
         <v/>
       </c>
-      <c r="H57" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>CVG</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>оценка; или встроенный плеер</t>
+          <t>все три зоны</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+          <t>CVGaudio VA-1100, регулятор «Зал» (100 Вт)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2240,7 +2252,7 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>2278</v>
+        <v>4246</v>
       </c>
       <c r="G58">
         <f>E58*F58</f>
@@ -2248,27 +2260,23 @@
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>Ozon</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>под iPad</t>
-        </is>
-      </c>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Шкаф</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
+          <t>CVGaudio VA-1100, регулятор «Улица» (100 Вт)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2280,7 +2288,7 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>17869</v>
+        <v>4246</v>
       </c>
       <c r="G59">
         <f>E59*F59</f>
@@ -2295,16 +2303,16 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CVGaudio OSR608TBL, зал 4 шт + улица 1 шт, 100 В</t>
+          <t>CVGaudio VA-110, регулятор «Туалет» (10 Вт)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2313,10 +2321,10 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>9417</v>
+        <v>2393</v>
       </c>
       <c r="G60">
         <f>E60*F60</f>
@@ -2331,92 +2339,92 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Акустика</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+          <t>Рамка / подрозетники под регуляторы</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>6150</v>
+        <v>1500</v>
       </c>
       <c r="G61">
         <f>E61*F61</f>
         <v/>
       </c>
-      <c r="H61" s="5" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>есть в наличии</t>
+          <t>оценка</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Кабель 2×1,5 (100 В), уличный кабель</t>
+          <t>iPad</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E62" t="n">
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="G62">
         <f>E62*F62</f>
         <v/>
       </c>
-      <c r="H62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Авито</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>примерно, нужен расчёт длины трасс</t>
+          <t>диапазон 17–25 тыс.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Расходные материалы (крепёж, коробки IP65)</t>
+          <t>Кабель/адаптер iPad → RCA</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2428,172 +2436,251 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="G63">
         <f>E63*F63</f>
         <v/>
       </c>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>оценка; или встроенный плеер</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="G64" s="4">
-        <f>SUM(G51:G63)</f>
-        <v/>
-      </c>
+      <c r="A64" t="n">
+        <v>8</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G64">
+        <f>E64*F64</f>
+        <v/>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>под iPad</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>9</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Шкаф</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>17869</v>
+      </c>
+      <c r="G65">
+        <f>E65*F65</f>
+        <v/>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>Вариант C: Lab.gruppen 100 В (CA2401 + CA602), сабвуфер опционально</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
-      <c r="H66" s="3" t="n"/>
-      <c r="I66" s="3" t="n"/>
+      <c r="A66" t="n">
+        <v>10</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>CVGaudio OSR608TBL, зал 4 шт + улица 1 шт, 100 В</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" t="n">
+        <v>9417</v>
+      </c>
+      <c r="G66">
+        <f>E66*F66</f>
+        <v/>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>Наименование</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>Цена, ₽</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>Сумма, ₽</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>Где купить</t>
-        </is>
-      </c>
-      <c r="I67" s="4" t="inlineStr">
-        <is>
-          <t>Примечание</t>
+      <c r="A67" t="n">
+        <v>11</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>6150</v>
+      </c>
+      <c r="G67">
+        <f>E67*F67</f>
+        <v/>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>CVG</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>есть в наличии</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Lab.gruppen CM82, микшер 8×2</t>
+          <t>Кабель 2×1,5 (100 В), уличный кабель</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E68" t="n">
         <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>45071</v>
+        <v>20000</v>
       </c>
       <c r="G68">
         <f>E68*F68</f>
         <v/>
       </c>
-      <c r="H68" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>примерно, нужен расчёт длины трасс</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA2401, зал (100 В)</t>
+          <t>Расходные материалы (крепёж, коробки IP65)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E69" t="n">
         <v>1</v>
       </c>
       <c r="F69" t="n">
-        <v>50100</v>
+        <v>7000</v>
       </c>
       <c r="G69">
         <f>E69*F69</f>
         <v/>
       </c>
-      <c r="H69" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
+      <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Lab.gruppen CA602, улица + туалет (100 В)</t>
+          <t>Кабель-канал DKC TA-GN 100×60 (01786), 2 м, под iPad и регуляторы, с перегородкой</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2602,10 +2689,10 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>44996</v>
+        <v>1150</v>
       </c>
       <c r="G70">
         <f>E70*F70</f>
@@ -2613,39 +2700,39 @@
       </c>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
+          <t>ВсеИнструменты</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>есть в наличии</t>
+          <t>перегородку и силовой выключатель уточнить, цена по выдаче поиска</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Lab.gruppen CRC-VEU, регулятор зоны</t>
+          <t>Заглушки DKC LAN 100×60 (00874), 2 шт</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>6510</v>
+        <v>191</v>
       </c>
       <c r="G71">
         <f>E71*F71</f>
@@ -2653,215 +2740,136 @@
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>зал, улица, туалет</t>
-        </is>
-      </c>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Электроника</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Рамка на 3 поста + подрозетники</t>
+          <t>Угол плоский DKC NPAN 100×60 (01745), поворот канала от шкафа к iPad</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E72" t="n">
         <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>1500</v>
+        <v>250</v>
       </c>
       <c r="G72">
         <f>E72*F72</f>
         <v/>
       </c>
-      <c r="H72" t="inlineStr"/>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>оценка</t>
+          <t>цена ориентировочно, уточнить</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="n">
-        <v>6</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Электроника</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>iPad</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>1</v>
-      </c>
-      <c r="F73" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G73">
-        <f>E73*F73</f>
-        <v/>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>Авито</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>диапазон 17–25 тыс.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="n">
-        <v>7</v>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Акустика</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>CVGaudio OSR608TBL, зал 4 шт (30 Вт) + улица 1 шт (20 Вт)</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E74" t="n">
-        <v>5</v>
-      </c>
-      <c r="F74" t="n">
-        <v>9417</v>
-      </c>
-      <c r="G74">
-        <f>E74*F74</f>
-        <v/>
-      </c>
-      <c r="H74" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G73" s="4">
+        <f>SUM(G57:G72)</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" t="n">
-        <v>8</v>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Акустика</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" t="n">
-        <v>6150</v>
-      </c>
-      <c r="G75">
-        <f>E75*F75</f>
-        <v/>
-      </c>
-      <c r="H75" s="5" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>есть в наличии</t>
-        </is>
-      </c>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Вариант C: Lab.gruppen 100 В (CA2401 + CA602), сабвуфер опционально</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="n"/>
+      <c r="C75" s="3" t="n"/>
+      <c r="D75" s="3" t="n"/>
+      <c r="E75" s="3" t="n"/>
+      <c r="F75" s="3" t="n"/>
+      <c r="G75" s="3" t="n"/>
+      <c r="H75" s="3" t="n"/>
+      <c r="I75" s="3" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" t="n">
-        <v>9</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Шкаф</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="E76" t="n">
-        <v>1</v>
-      </c>
-      <c r="F76" t="n">
-        <v>17869</v>
-      </c>
-      <c r="G76">
-        <f>E76*F76</f>
-        <v/>
-      </c>
-      <c r="H76" s="5" t="inlineStr">
-        <is>
-          <t>Pult.ru</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Блок розеток 19″ 1U с выключателем MDX PDU-8E-10A-Sw</t>
+          <t>Lab.gruppen CM82, микшер 8×2</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2873,7 +2881,7 @@
         <v>1</v>
       </c>
       <c r="F77" t="n">
-        <v>2080</v>
+        <v>45071</v>
       </c>
       <c r="G77">
         <f>E77*F77</f>
@@ -2888,16 +2896,16 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+          <t>Lab.gruppen CA2401, зал (100 В)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2909,7 +2917,7 @@
         <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>2278</v>
+        <v>50100</v>
       </c>
       <c r="G78">
         <f>E78*F78</f>
@@ -2917,172 +2925,255 @@
       </c>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>Ozon</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>под iPad</t>
-        </is>
-      </c>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
+          <t>Lab.gruppen CA602, улица + туалет (100 В)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>20000</v>
+        <v>44996</v>
       </c>
       <c r="G79">
         <f>E79*F79</f>
         <v/>
       </c>
-      <c r="H79" t="inlineStr"/>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>примерно, нужен расчёт длины трасс</t>
+          <t>есть в наличии</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Шкаф и материалы</t>
+          <t>Электроника</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Расходные материалы</t>
+          <t>Lab.gruppen CRC-VEU, регулятор зоны</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F80" t="n">
-        <v>8000</v>
+        <v>6510</v>
       </c>
       <c r="G80">
         <f>E80*F80</f>
         <v/>
       </c>
-      <c r="H80" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
       <c r="I80" t="inlineStr">
         <is>
+          <t>зал, улица, туалет</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>5</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Рамка на 3 поста + подрозетники</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G81">
+        <f>E81*F81</f>
+        <v/>
+      </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
           <t>оценка</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="G81" s="4">
-        <f>SUM(G68:G80)</f>
-        <v/>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>6</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Электроника</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>iPad</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G82">
+        <f>E82*F82</f>
+        <v/>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Авито</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>диапазон 17–25 тыс.</t>
+        </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>Вариант C: опция «сабвуфер»</t>
-        </is>
-      </c>
-      <c r="B83" s="3" t="n"/>
-      <c r="C83" s="3" t="n"/>
-      <c r="D83" s="3" t="n"/>
-      <c r="E83" s="3" t="n"/>
-      <c r="F83" s="3" t="n"/>
-      <c r="G83" s="3" t="n"/>
-      <c r="H83" s="3" t="n"/>
-      <c r="I83" s="3" t="n"/>
+      <c r="A83" t="n">
+        <v>7</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CVGaudio OSR608TBL, зал 4 шт (30 Вт) + улица 1 шт (20 Вт)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>5</v>
+      </c>
+      <c r="F83" t="n">
+        <v>9417</v>
+      </c>
+      <c r="G83">
+        <f>E83*F83</f>
+        <v/>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B84" s="4" t="inlineStr">
-        <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>Наименование</t>
-        </is>
-      </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-      <c r="F84" s="4" t="inlineStr">
-        <is>
-          <t>Цена, ₽</t>
-        </is>
-      </c>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>Сумма, ₽</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="inlineStr">
-        <is>
-          <t>Где купить</t>
-        </is>
-      </c>
-      <c r="I84" s="4" t="inlineStr">
-        <is>
-          <t>Примечание</t>
+      <c r="A84" t="n">
+        <v>8</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Акустика</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CVGaudio CRH608T, туалет, 100 В / 8 Вт</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="n">
+        <v>6150</v>
+      </c>
+      <c r="G84">
+        <f>E84*F84</f>
+        <v/>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>CVG</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>есть в наличии</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Опция</t>
+          <t>Шкаф</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Усилитель мощности Behringer KM750</t>
+          <t>Шкаф настенный 19″ 9U Wize Pro W9U45R</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3094,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="F85" t="n">
-        <v>21475</v>
+        <v>17869</v>
       </c>
       <c r="G85">
         <f>E85*F85</f>
@@ -3105,24 +3196,20 @@
           <t>Pult.ru</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>канал под сабвуфер</t>
-        </is>
-      </c>
+      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Опция</t>
+          <t>Шкаф и материалы</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
+          <t>Блок розеток 19″ 1U с выключателем MDX PDU-8E-10A-Sw</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3134,7 +3221,7 @@
         <v>1</v>
       </c>
       <c r="F86" t="n">
-        <v>49990</v>
+        <v>2080</v>
       </c>
       <c r="G86">
         <f>E86*F86</f>
@@ -3142,19 +3229,396 @@
       </c>
       <c r="H86" s="5" t="inlineStr">
         <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>11</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Кронштейн настенный металлический для планшетов 4–13″</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G87">
+        <f>E87*F87</f>
+        <v/>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>под iPad</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>12</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Кабель: 2×1,5 (100 В), уличный, Cat5e ×3, 2×2,5 под саб</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G88">
+        <f>E88*F88</f>
+        <v/>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>примерно, нужен расчёт длины трасс</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>13</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Расходные материалы</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G89">
+        <f>E89*F89</f>
+        <v/>
+      </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>оценка</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>14</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Кабель-канал DKC TA-GN 100×60 (01786), 2 м, под iPad и регуляторы, с перегородкой</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="n">
+        <v>1150</v>
+      </c>
+      <c r="G90">
+        <f>E90*F90</f>
+        <v/>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>перегородку и силовой выключатель уточнить, цена по выдаче поиска</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>15</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Заглушки DKC LAN 100×60 (00874), 2 шт</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" t="n">
+        <v>191</v>
+      </c>
+      <c r="G91">
+        <f>E91*F91</f>
+        <v/>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>16</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Шкаф и материалы</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Угол плоский DKC NPAN 100×60 (01745), поворот канала от шкафа к iPad</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" t="n">
+        <v>250</v>
+      </c>
+      <c r="G92">
+        <f>E92*F92</f>
+        <v/>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>ВсеИнструменты</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>цена ориентировочно, уточнить</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="G93" s="4">
+        <f>SUM(G77:G92)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Вариант C: опция «сабвуфер»</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="n"/>
+      <c r="C95" s="3" t="n"/>
+      <c r="D95" s="3" t="n"/>
+      <c r="E95" s="3" t="n"/>
+      <c r="F95" s="3" t="n"/>
+      <c r="G95" s="3" t="n"/>
+      <c r="H95" s="3" t="n"/>
+      <c r="I95" s="3" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Цена, ₽</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>Сумма, ₽</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>Где купить</t>
+        </is>
+      </c>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>1</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Опция</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Усилитель мощности Behringer KM750</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="n">
+        <v>21475</v>
+      </c>
+      <c r="G97">
+        <f>E97*F97</f>
+        <v/>
+      </c>
+      <c r="H97" s="5" t="inlineStr">
+        <is>
+          <t>Pult.ru</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>канал под сабвуфер</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>2</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Опция</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Radiotehnika Alfa 1.04 MKII, активный сабвуфер 10″</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="n">
+        <v>49990</v>
+      </c>
+      <c r="G98">
+        <f>E98*F98</f>
+        <v/>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
           <t>Audiomania</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="C87" s="4" t="inlineStr">
+      <c r="I98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
       </c>
-      <c r="G87" s="4">
-        <f>SUM(G85:G86)</f>
+      <c r="G99" s="4">
+        <f>SUM(G97:G98)</f>
         <v/>
       </c>
     </row>
@@ -3170,37 +3634,49 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>